<commit_message>
Remove Marco Sanna duplicate from contacts.xlsx
Marco Sanna already exists in attendees.xlsx from the previous session;
drop the duplicate so contacts.xlsx contains only new entries.

https://claude.ai/code/session_01Dy4Y591rmUgrFA1cD8J2m3
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1352,45 +1352,32 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Marco Sanna</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
+          <t>KATSUYUKI SHINZEKI</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Assistant Manager</t>
+        </is>
+      </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>cbs Corporate Business Solutions Unternehm...</t>
+          <t>Marubeni Corporation</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>KATSUYUKI SHINZEKI</t>
+          <t>JASBIR SINGH</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Assistant Manager</t>
+          <t>Associate Partner, Global...</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
-        <is>
-          <t>Marubeni Corporation</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>JASBIR SINGH</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Associate Partner, Global...</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
         <is>
           <t>IBM India Pvt Ltd</t>
         </is>

</xml_diff>